<commit_message>
Update Errors across files
</commit_message>
<xml_diff>
--- a/Files List Error Tracking.xlsx
+++ b/Files List Error Tracking.xlsx
@@ -8,19 +8,42 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AppDev\DebitLens\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7E03E24-364A-47FC-94DB-DDB00EF05D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{63CDCEC1-4EAC-42A0-AFA6-37C4D4DF03E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{0EC2DA8C-4978-4A72-B938-F974F5269E45}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{0EC2DA8C-4978-4A72-B938-F974F5269E45}"/>
   </bookViews>
   <sheets>
-    <sheet name="Files List" sheetId="1" r:id="rId1"/>
+    <sheet name="Error List" sheetId="2" r:id="rId1"/>
+    <sheet name="Files List" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="88">
   <si>
     <t>AccountForm.tsx"</t>
   </si>
@@ -284,27 +307,6 @@
   </si>
   <si>
     <t>Errors</t>
-  </si>
-  <si>
-    <t>Property 'prefs' does not exist on type 'AppState'.
-Property 'prefs' does not exist on type 'AppState'.</t>
-  </si>
-  <si>
-    <t>Property 'label' does not exist on type 'Account'.
-Object literal may only specify known properties, and 'label' does not exist in type 'Partial&lt;Account&gt;'.</t>
-  </si>
-  <si>
-    <t>Property 'note' does not exist on type 'Transaction'.</t>
-  </si>
-  <si>
-    <t>Object literal may only specify known properties, and 'label' does not exist in type 'Partial&lt;Account&gt;'.</t>
-  </si>
-  <si>
-    <t>Module '"../state/AppContext"' has no exported member 'Budget'.
-Property 'budgets' does not exist on type 'AppState'.
-Property 'updateBudget' does not exist on type 'AppActions'.
-Property 'addBudget' does not exist on type 'AppActions'.
-Property 'deleteBudget' does not exist on type 'AppActions'.</t>
   </si>
 </sst>
 </file>
@@ -794,8 +796,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1185,789 +1194,804 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C0B799D-B152-4EDC-90BC-C1450490B7CC}">
+  <dimension ref="A2:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="114.5703125" style="3" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="str" cm="1">
+        <f t="array" ref="A2:D2">_xlfn._xlws.FILTER('Files List'!A:D, 'Files List'!D:D&lt;&gt;"")</f>
+        <v>Root Folder</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>Sub Folder</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>Files</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Errors</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:4" ht="75" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:4" ht="120" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:4" ht="150" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="60" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41C8E12-756B-4D03-AF8C-7EAD0401066F}">
   <dimension ref="A1:D68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="73.5703125" style="5" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="22.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.5703125" style="8" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" s="5" t="s">
+      <c r="A2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B17" s="5" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B18" s="5" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B19" s="5" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" s="5" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="5" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="5" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="5" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B24" s="5" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="5" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="5" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C27" s="5" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="5" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" s="5" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C30" s="5" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C31" s="5" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="5" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="5" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="5" t="s">
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" s="5" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C36" s="5" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C37" s="5" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C38" s="5" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39" s="5" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" s="5" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" s="5" t="s">
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="5" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" s="5" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" s="5" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" s="5" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46" s="5" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C47" s="5" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C48" s="5" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C49" s="5" t="s">
+      <c r="A49" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C50" s="5" t="s">
+      <c r="A50" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B51" s="5" t="s">
+      <c r="A51" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B52" s="5" t="s">
+      <c r="A52" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="8" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B53" s="5" t="s">
+      <c r="A53" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B54" s="5" t="s">
+      <c r="A54" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="8" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B55" s="5" t="s">
+      <c r="A55" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B55" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="8" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B56" s="5" t="s">
+      <c r="A56" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B56" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="8" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B57" s="5" t="s">
+      <c r="A57" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B57" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C57" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B58" s="5" t="s">
+      <c r="A58" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="8" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B59" s="5" t="s">
+      <c r="A59" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B59" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C59" s="8" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B60" s="5" t="s">
+      <c r="A60" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B61" s="5" t="s">
+      <c r="A61" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B61" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="8" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B62" s="5" t="s">
+      <c r="A62" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="8" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B63" s="5" t="s">
+      <c r="A63" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B63" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="C63" s="8" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B64" s="5" t="s">
+      <c r="A64" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="C64" s="8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B65" s="5" t="s">
+      <c r="A65" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" s="8" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
+      <c r="A66" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B66" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C66" s="5" t="s">
+      <c r="B66" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B67" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C67" s="5" t="s">
+      <c r="B67" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="4" t="s">
+      <c r="A68" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="C68" s="8" t="s">
         <v>82</v>
       </c>
     </row>

</xml_diff>